<commit_message>
Auth: login por usuario/contraseña, roles y esquema de base de datos
- supabase/migrations/0001_init.sql: tablas (profiles, employees,
  weekly_schedules, qr_tokens, time_entries, hour_adjustments,
  audit_log), función is_owner() y políticas RLS de solo lectura (las
  escrituras se hacen siempre desde el servidor con la service role key).
- lib/supabase/{server,client,admin}.ts: helpers de @supabase/ssr para
  Server Components, Client Components y operaciones administrativas.
- middleware.ts: refresca la sesión y redirige según rol (dueño -> /admin,
  empleado -> /), protegiendo /admin del lado del servidor.
- /login: resuelve usuario -> email y autentica con Supabase Auth (RF-01,
  RF-02). /auth/callback + /set-password: define la contraseña personal
  a partir del enlace de invitación (RF-23).
- Backlog: RF-01 y RF-02 marcados Completado (falta correr la migración
  SQL en el proyecto real de Supabase para probarlo en vivo).
</commit_message>
<xml_diff>
--- a/Backlog_Requerimientos_Control_Horario_Cafeteria.xlsx
+++ b/Backlog_Requerimientos_Control_Horario_Cafeteria.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="157">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -488,6 +488,15 @@
   </si>
   <si>
     <t xml:space="preserve">El propio sistema de autenticación de Supabase permite enviar automáticamente el correo de bienvenida con el enlace para que el empleado configure su contraseña, sin necesidad de contratar un servicio de correo por separado.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Completado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login por usuario+contraseña (resuelve usuario a email y usa Supabase Auth). Falta correr supabase/migrations/0001_init.sql en el proyecto real para probarlo en vivo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mismo login que RF-01; el middleware redirige a /admin cuando el rol es dueño. Falta correr la migración SQL para probarlo en vivo.</t>
   </si>
 </sst>
 </file>
@@ -1030,9 +1039,11 @@
         <v>11</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G2" s="2"/>
+        <v>154</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>155</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
@@ -1051,9 +1062,11 @@
         <v>16</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="G3" s="4"/>
+        <v>154</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>156</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">

</xml_diff>

<commit_message>
Gestión de empleados: alta, edición, username automático e invitación
- lib/username.ts: genera el usuario (primera letra del nombre +
  apellido, sin acentos/espacios) con desambiguación incremental ante
  colisión (regla 13, RF-21). Tests unitarios en
  lib/__tests__/username.test.ts.
- app/admin/empleados: listado, alta (invita por correo con
  supabase.auth.admin.inviteUserByEmail, RF-22), edición de datos
  obligatorios (RF-08), reenvío de invitación (RF-24) y
  activar/desactivar empleado.
- lib/audit.ts + lib/auth/current-user.ts: helpers reutilizables para
  dejar trazabilidad de altas/ediciones en audit_log (RF-19).
- vitest.config.ts: alias @/ para los tests.
- Backlog: RF-08, RF-21, RF-22, RF-23, RF-24 marcados Completado.
</commit_message>
<xml_diff>
--- a/Backlog_Requerimientos_Control_Horario_Cafeteria.xlsx
+++ b/Backlog_Requerimientos_Control_Horario_Cafeteria.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="162">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -497,6 +497,21 @@
   </si>
   <si>
     <t xml:space="preserve">Mismo login que RF-01; el middleware redirige a /admin cuando el rol es dueño. Falta correr la migración SQL para probarlo en vivo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alta/edición/desactivación de empleados en /admin/empleados. Falta correr la migración SQL para probar en vivo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lib/username.ts genera el usuario (primera letra + apellido, sin acentos) con desambiguación por colisión. Cubierto por tests unitarios.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Al crear el empleado se invita por correo con supabase.auth.admin.inviteUserByEmail. Falta probarlo con el proyecto real.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/set-password permite al empleado definir su contraseña vía el enlace de invitación; el dueño nunca la ve.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Botón "Reenviar invitación" en /admin/empleados/[id].</t>
   </si>
 </sst>
 </file>
@@ -1190,9 +1205,11 @@
         <v>16</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="G9" s="4"/>
+        <v>154</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>157</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="90.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
@@ -1463,9 +1480,11 @@
         <v>24</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G22" s="2"/>
+        <v>154</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>158</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
@@ -1484,9 +1503,11 @@
         <v>24</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="G23" s="4"/>
+        <v>154</v>
+      </c>
+      <c r="G23" s="4" t="s">
+        <v>159</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
@@ -1505,9 +1526,11 @@
         <v>11</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G24" s="2"/>
+        <v>154</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
@@ -1526,9 +1549,11 @@
         <v>16</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="G25" s="4"/>
+        <v>154</v>
+      </c>
+      <c r="G25" s="4" t="s">
+        <v>161</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:G25"/>

</xml_diff>

<commit_message>
Horario semanal por empleado y vista informativa (RF-09, RF-07)
- lib/week.ts: cálculo de semana lunes-domingo en huso America/Montevideo.
- lib/schedule.ts: horas totales por día/semana y resolución del horario
  vigente (override semanal si existe, si no el horario por defecto del
  empleado), con tests unitarios.
- components/schedule-days-editor.tsx: editor de días/horas reutilizable
  (checkbox + horario) con total sugerido en vivo.
- /admin/empleados/[id]/horario: edición del horario de la semana en
  curso (con navegación entre semanas) y del horario por defecto del
  empleado.
- Home del empleado: agrega la vista de solo lectura del horario
  acordado de la semana en curso.
- Backlog: RF-09 y RF-07 marcados Completado.
</commit_message>
<xml_diff>
--- a/Backlog_Requerimientos_Control_Horario_Cafeteria.xlsx
+++ b/Backlog_Requerimientos_Control_Horario_Cafeteria.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="164">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -512,6 +512,12 @@
   </si>
   <si>
     <t xml:space="preserve">Botón "Reenviar invitación" en /admin/empleados/[id].</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El home del empleado muestra el horario acordado de la semana en curso (solo informativo).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/admin/empleados/[id]/horario: editor por semana (lunes a domingo) con total de horas sugerido en vivo, navegación entre semanas y horario por defecto reutilizable.</t>
   </si>
 </sst>
 </file>
@@ -1184,9 +1190,11 @@
         <v>11</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G8" s="2"/>
+        <v>154</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>162</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="90.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
@@ -1228,9 +1236,11 @@
         <v>16</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G10" s="2"/>
+        <v>154</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>163</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">

</xml_diff>

<commit_message>
QR maestro: generación, descarga y regeneración (RF-18)
- lib/qr.ts: token activo único (qr_tokens), genera/descarga la imagen
  PNG del QR (paquete qrcode) y regenera invalidando el anterior, con
  auditoría.
- /admin/qr: muestra el QR vigente, botón de descarga y regeneración
  con confirmación (evita invalidar el QR impreso por error).
- app/admin/layout.tsx: fuerza renderizado dinámico en todo el panel
  del dueño (`export const dynamic = "force-dynamic"`) — sin este
  cambio, Next intentaba pre-renderizar /admin/qr en build time y
  ensureQrToken() (que puede crear el primer token) se ejecutaba contra
  Supabase durante el build en lugar de en tiempo de request.
- Backlog: RF-18 marcado Completado.
</commit_message>
<xml_diff>
--- a/Backlog_Requerimientos_Control_Horario_Cafeteria.xlsx
+++ b/Backlog_Requerimientos_Control_Horario_Cafeteria.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="165">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -518,6 +518,9 @@
   </si>
   <si>
     <t xml:space="preserve">/admin/empleados/[id]/horario: editor por semana (lunes a domingo) con total de horas sugerido en vivo, navegación entre semanas y horario por defecto reutilizable.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/admin/qr genera, descarga y regenera el QR maestro (invalida el anterior y deja auditoría). Falta correr la migración SQL para probarlo en vivo.</t>
   </si>
 </sst>
 </file>
@@ -1427,9 +1430,11 @@
         <v>67</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="G19" s="4"/>
+        <v>154</v>
+      </c>
+      <c r="G19" s="4" t="s">
+        <v>164</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">

</xml_diff>

<commit_message>
Marcado de entrada/salida con escaneo de QR en la app (RF-03, RF-04, RF-05)
- lib/attendance/pairing.ts: empareja tramos entrada/salida del día y
  determina el próximo tipo de marca (RF-04), con tests unitarios que
  cubren tramos múltiples y jornadas abiertas.
- lib/attendance/daily.ts: marcas y total del día calendario en
  America/Montevideo, reutilizado por el home del empleado (RF-05).
- lib/attendance/mark.ts + /api/time-entries/mark: valida el QR
  escaneado contra el token activo (lib/qr.ts) y registra la marca
  (RF-03).
- /marcar: activa la cámara con html5-qrcode, confirma la marca y
  vuelve al home mostrando la hora registrada.
- Home del empleado: botón único "Marcar entrada/salida" (según el
  próximo tipo detectado), listado de marcas de hoy y total del día.
- lib/week.ts: agrega límites de día/semana en huso horario local,
  reutilizables para el saldo semanal.
- Backlog: RF-03, RF-04 y RF-05 marcados Completado.
</commit_message>
<xml_diff>
--- a/Backlog_Requerimientos_Control_Horario_Cafeteria.xlsx
+++ b/Backlog_Requerimientos_Control_Horario_Cafeteria.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="168">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -521,6 +521,15 @@
   </si>
   <si>
     <t xml:space="preserve">/admin/qr genera, descarga y regenera el QR maestro (invalida el anterior y deja auditoría). Falta correr la migración SQL para probarlo en vivo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/marcar activa la cámara (html5-qrcode), valida el QR contra el token activo y registra la marca en /api/time-entries/mark. Falta correr la migración SQL para probarlo en vivo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lib/attendance/pairing.ts determina entrada/salida según las marcas del día (con tests unitarios).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Home del empleado: marcas del día y total (lib/attendance/daily.ts).</t>
   </si>
 </sst>
 </file>
@@ -1109,9 +1118,11 @@
         <v>11</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G4" s="2"/>
+        <v>154</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>165</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
@@ -1130,9 +1141,11 @@
         <v>24</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="G5" s="4"/>
+        <v>154</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>166</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
@@ -1151,9 +1164,11 @@
         <v>11</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G6" s="2"/>
+        <v>154</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>167</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">

</xml_diff>

<commit_message>
Saldo semanal del empleado (RF-06, RF-13, RF-14)
- lib/attendance/balance-math.ts: cálculo puro del saldo (pactadas -
  trabajadas + ajustes), con tests unitarios.
- lib/attendance/balance.ts: obtiene marcas y ajustes de la semana
  (huso America/Montevideo) y arma el saldo real.
- Home del empleado: sección de saldo semanal (pactadas, trabajadas,
  ajustes si aplica, saldo con color según signo).
- Backlog: RF-06, RF-13 y RF-14 marcados Completado.
</commit_message>
<xml_diff>
--- a/Backlog_Requerimientos_Control_Horario_Cafeteria.xlsx
+++ b/Backlog_Requerimientos_Control_Horario_Cafeteria.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="171">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -530,6 +530,15 @@
   </si>
   <si>
     <t xml:space="preserve">Home del empleado: marcas del día y total (lib/attendance/daily.ts).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Home del empleado muestra pactadas, trabajadas, ajustes y saldo de la semana en curso.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lib/attendance/pairing.ts suma los tramos del día al minuto exacto (sin redondeo).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lib/attendance/balance.ts calcula el saldo semanal (pactadas - trabajadas + ajustes) en tiempo real, con tests unitarios.</t>
   </si>
 </sst>
 </file>
@@ -1187,9 +1196,11 @@
         <v>11</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="G7" s="4"/>
+        <v>154</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>168</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
@@ -1340,9 +1351,11 @@
         <v>24</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G14" s="2"/>
+        <v>154</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>169</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
@@ -1361,9 +1374,11 @@
         <v>24</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="G15" s="4"/>
+        <v>154</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>170</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">

</xml_diff>

<commit_message>
Panel de marcas del dueño: filtros, pendientes y corrección manual
- lib/attendance/review-math.ts: agrupa marcas por empleado/día y
  marca "pendiente de revisión" los días pasados con una entrada sin
  salida (regla de negocio 1), con tests unitarios.
- lib/attendance/review.ts: trae las marcas de Supabase para un rango
  de fechas y arma los grupos.
- /admin/marcas: filtro por empleado y rango de fechas (cualquier
  período pasado, RF-17), listado agrupado por día con badge de
  pendiente de revisión (RF-11), edición inline y eliminación de
  marcas, y alta manual (RF-12) — todo deja auditoría en audit_log
  (RF-19).
- lib/week.ts: agrega helpers de rango de fechas y formato de
  hora/input local reutilizados por el panel.
- Backlog: RF-10, RF-11, RF-12, RF-17 y RF-19 marcados Completado.
</commit_message>
<xml_diff>
--- a/Backlog_Requerimientos_Control_Horario_Cafeteria.xlsx
+++ b/Backlog_Requerimientos_Control_Horario_Cafeteria.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="176">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -539,6 +539,21 @@
   </si>
   <si>
     <t xml:space="preserve">lib/attendance/balance.ts calcula el saldo semanal (pactadas - trabajadas + ajustes) en tiempo real, con tests unitarios.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/admin/marcas: listado filtrable por empleado y rango de fechas, agrupado por día.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Días pasados con una entrada sin salida se marcan "Pendiente de revisión" (no se contabilizan hasta corregirse).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Edición inline (tipo/hora/nota), eliminación y alta manual de marcas, todas identificadas como manuales en el historial.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El mismo panel de marcas permite elegir cualquier rango de fechas pasado.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Toda alta/edición/borrado manual de marcas queda en audit_log (lib/audit.ts) con actor, valor anterior y nuevo.</t>
   </si>
 </sst>
 </file>
@@ -1288,9 +1303,11 @@
         <v>16</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="G11" s="4"/>
+        <v>154</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>171</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
@@ -1309,9 +1326,11 @@
         <v>24</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G12" s="2"/>
+        <v>154</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>172</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="102.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
@@ -1330,9 +1349,11 @@
         <v>16</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="G13" s="4"/>
+        <v>154</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>173</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
@@ -1439,9 +1460,11 @@
         <v>16</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G18" s="2"/>
+        <v>154</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>174</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="77.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
@@ -1483,9 +1506,11 @@
         <v>24</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G20" s="2"/>
+        <v>154</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>175</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">

</xml_diff>

<commit_message>
Ajustes manuales de horas (RF-15)
- /admin/ajustes: alta de ajuste (empleado, semana, horas +/-, concepto
  libre) y eliminación, con auditoría (audit_log). El ajuste ya se
  refleja en el saldo semanal del empleado porque lib/attendance/balance.ts
  suma hour_adjustments por (employee_id, week_start).
- Backlog: RF-15 marcado Completado.
</commit_message>
<xml_diff>
--- a/Backlog_Requerimientos_Control_Horario_Cafeteria.xlsx
+++ b/Backlog_Requerimientos_Control_Horario_Cafeteria.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="177">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -554,6 +554,9 @@
   </si>
   <si>
     <t xml:space="preserve">Toda alta/edición/borrado manual de marcas queda en audit_log (lib/audit.ts) con actor, valor anterior y nuevo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/admin/ajustes: alta (empleado, semana, horas +/-, concepto libre) y eliminación, ya integrado al cálculo de saldo semanal. Falta correr la migración SQL para probarlo en vivo.</t>
   </si>
 </sst>
 </file>
@@ -1418,9 +1421,11 @@
         <v>16</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G16" s="2"/>
+        <v>154</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>176</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">

</xml_diff>

<commit_message>
Reporte mensual en Excel para liquidación de haberes (RF-16)
- lib/reports/monthly-math.ts: asigna cada semana (lunes a domingo) al
  mes en que empieza, y genera nombres de hoja de Excel válidos/únicos
  por empleado, con tests unitarios.
- lib/reports/monthly.ts: arma el workbook (exceljs) con una hoja
  "Consolidado" (todas las semanas de todos los empleados + totales del
  mes) y una hoja por empleado, reutilizando lib/attendance/balance.ts.
- /api/reports/monthly: ruta protegida (solo dueño) que devuelve el
  .xlsx como descarga.
- /admin/reportes: selector de mes + descarga.
- Backlog: RF-16 marcado Completado.
</commit_message>
<xml_diff>
--- a/Backlog_Requerimientos_Control_Horario_Cafeteria.xlsx
+++ b/Backlog_Requerimientos_Control_Horario_Cafeteria.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="178">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -557,6 +557,9 @@
   </si>
   <si>
     <t xml:space="preserve">/admin/ajustes: alta (empleado, semana, horas +/-, concepto libre) y eliminación, ya integrado al cálculo de saldo semanal. Falta correr la migración SQL para probarlo en vivo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/admin/reportes + /api/reports/monthly genera un .xlsx (consolidado + una hoja por empleado) con horas, saldos semanales, ajustes y totales del mes. PDF queda como mejora futura. Falta correr la migración SQL para probarlo en vivo.</t>
   </si>
 </sst>
 </file>
@@ -1444,9 +1447,11 @@
         <v>16</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="G17" s="4"/>
+        <v>154</v>
+      </c>
+      <c r="G17" s="4" t="s">
+        <v>177</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">

</xml_diff>

<commit_message>
Confirmar en vivo el fix de RF-16 (reporte mensual)
El usuario confirmó que, tras el fix de semanas superpuestas, el
reporte de julio ya muestra correctamente las horas trabajadas y el
ajuste de Ana Rodriguez.
</commit_message>
<xml_diff>
--- a/Backlog_Requerimientos_Control_Horario_Cafeteria.xlsx
+++ b/Backlog_Requerimientos_Control_Horario_Cafeteria.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="194">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -605,6 +605,9 @@
   </si>
   <si>
     <t xml:space="preserve">Verificado en vivo: se ve el QR y se descarga correctamente. Falta probar el botón de regenerar.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verificado en vivo tras corregir el bug de semanas superpuestas: el reporte de julio ya muestra correctamente las horas trabajadas y el ajuste de Ana. Ver ESTADO_PRUEBAS.md.</t>
   </si>
 </sst>
 </file>
@@ -1495,7 +1498,7 @@
         <v>154</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Actualizar estado de pruebas: RF-07, RF-09, RF-11, RF-17, RF-19
Registro de lo verificado en vivo en esta ronda: vista de horario del
empleado, editor de horario semanal (con el bug de estado stale
encontrado y corregido), alerta de pendiente de revisión, filtro de
fechas del panel de marcas, y auditoría de correcciones.
</commit_message>
<xml_diff>
--- a/Backlog_Requerimientos_Control_Horario_Cafeteria.xlsx
+++ b/Backlog_Requerimientos_Control_Horario_Cafeteria.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="199">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -608,6 +608,21 @@
   </si>
   <si>
     <t xml:space="preserve">Verificado en vivo tras corregir el bug de semanas superpuestas: el reporte de julio ya muestra correctamente las horas trabajadas y el ajuste de Ana. Ver ESTADO_PRUEBAS.md.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verificado en vivo: el empleado ve el horario acordado actualizado en su home.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se encontró y corrigió un bug real en vivo: el editor conservaba datos de la semana/empleado anterior al navegar. Ver ESTADO_PRUEBAS.md.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verificado en vivo: el cartel de pendiente de revisión aparece correctamente para una marca sin salida de un día pasado.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verificado en vivo: el filtro de fecha del panel de marcas muestra correctamente marcas fuera de la semana en curso.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verificado por script directo: audit_log registra correctamente las acciones con actor y valores anterior/nuevo.</t>
   </si>
 </sst>
 </file>
@@ -1291,7 +1306,7 @@
         <v>154</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>162</v>
+        <v>194</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="90.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1337,7 +1352,7 @@
         <v>154</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>163</v>
+        <v>195</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1383,7 +1398,7 @@
         <v>154</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>172</v>
+        <v>196</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="102.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1521,7 +1536,7 @@
         <v>154</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>174</v>
+        <v>197</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="77.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1567,7 +1582,7 @@
         <v>154</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>175</v>
+        <v>198</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Actualizar estado de pruebas: bug de RF-18 documentado
</commit_message>
<xml_diff>
--- a/Backlog_Requerimientos_Control_Horario_Cafeteria.xlsx
+++ b/Backlog_Requerimientos_Control_Horario_Cafeteria.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="200">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -623,6 +623,9 @@
   </si>
   <si>
     <t xml:space="preserve">Verificado por script directo: audit_log registra correctamente las acciones con actor y valores anterior/nuevo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se encontró y corrigió de raíz una condición de carrera real (rompía /admin/qr) moviendo la regeneración del QR a una función atómica en Postgres. Ver ESTADO_PRUEBAS.md. Falta reconfirmar en vivo.</t>
   </si>
 </sst>
 </file>
@@ -1559,7 +1562,7 @@
         <v>154</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>192</v>
+        <v>199</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Confirmar en vivo el fix de RF-18 (QR maestro)
El usuario confirmó, tras un hard refresh, que /admin/qr carga
correctamente y el botón "Regenerar QR" funciona. El error persistía
por un overlay de error cacheado en el navegador tras reiniciar el
servidor, no por el código.
</commit_message>
<xml_diff>
--- a/Backlog_Requerimientos_Control_Horario_Cafeteria.xlsx
+++ b/Backlog_Requerimientos_Control_Horario_Cafeteria.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="201">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -626,6 +626,9 @@
   </si>
   <si>
     <t xml:space="preserve">Se encontró y corrigió de raíz una condición de carrera real (rompía /admin/qr) moviendo la regeneración del QR a una función atómica en Postgres. Ver ESTADO_PRUEBAS.md. Falta reconfirmar en vivo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se encontró y corrigió de raíz una condición de carrera real (rompía /admin/qr) moviendo la regeneración del QR a una función atómica en Postgres. Confirmado en vivo: la página y el botón de regenerar funcionan correctamente.</t>
   </si>
 </sst>
 </file>
@@ -1562,7 +1565,7 @@
         <v>154</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Actualizar seguimiento de RF-08/RF-16 con valor hora y liquidacion
Refleja en el backlog y en ESTADO_PRUEBAS.md que se agrego el campo
valor hora nominal y la liquidacion mensual con detalle diario,
pendientes de reconfirmar en vivo.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Backlog_Requerimientos_Control_Horario_Cafeteria.xlsx
+++ b/Backlog_Requerimientos_Control_Horario_Cafeteria.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="205">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -629,6 +629,18 @@
   </si>
   <si>
     <t xml:space="preserve">Se encontró y corrigió de raíz una condición de carrera real (rompía /admin/qr) moviendo la regeneración del QR a una función atómica en Postgres. Confirmado en vivo: la página y el botón de regenerar funcionan correctamente.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El dueño puede crear, editar y desactivar empleados. Al crear un empleado, debe ingresar: nombre completo, cédula, teléfono de contacto, mutualista, contacto de emergencia y correo electrónico (obligatorio, utilizado para el acceso y las comunicaciones del sistema), además de su cantidad de horas semanales pactadas, su valor hora nominal (obligatorio, usado para calcular la liquidación mensual) y un horario por defecto (días/horas), que se usará como base al configurar la semana en curso.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verificado en vivo desde la app real: alta de empleado, generación de usuario e invitación por correo confirmadas. Se agregó el campo obligatorio "Valor hora nominal" (migración 0003_employee_hourly_rate.sql, ya aplicada a la base real). Falta reconfirmar en vivo el alta/edición con el campo nuevo — ver ESTADO_PRUEBAS.md.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El sistema genera un reporte descargable (Excel/PDF) por empleado y consolidado, con horas trabajadas, saldos semanales, ajustes manuales aplicados y totales del mes, listo para liquidación de haberes. Incluye el cálculo de la liquidación mensual (horas hasta las pactadas a valor simple, excedente pagado al doble, con las "horas extras que se están pagando" explícitas) y, en la hoja de cada empleado, un detalle diario de entrada/salida/horas trabajadas además del resumen semanal.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verificado en vivo tras corregir el bug de semanas superpuestas: el reporte de julio ya muestra correctamente las horas trabajadas y el ajuste de Ana. Se agregó la liquidación mensual y el detalle diario por empleado (8 tests unitarios nuevos en monthly-math.test.ts); falta descargar un reporte real y confirmar visualmente ambas secciones nuevas. Ver ESTADO_PRUEBAS.md.</t>
   </si>
 </sst>
 </file>
@@ -1323,7 +1335,7 @@
         <v>35</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>36</v>
+        <v>201</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>10</v>
@@ -1335,7 +1347,7 @@
         <v>154</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>180</v>
+        <v>202</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="90.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1507,7 +1519,7 @@
         <v>59</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>60</v>
+        <v>203</v>
       </c>
       <c r="D17" s="5" t="s">
         <v>10</v>
@@ -1519,7 +1531,7 @@
         <v>154</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>193</v>
+        <v>204</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Confirmar RF-03 en produccion y documentar despliegue en Vercel
Usuario confirmo desde el celular, en produccion (Vercel, HTTPS): login,
carga de la app y marcado real de entrada/salida por camara/QR
funcionando correctamente. Esto cierra la unica prueba que habia
quedado pendiente por el requisito de HTTPS para acceso a camara.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Backlog_Requerimientos_Control_Horario_Cafeteria.xlsx
+++ b/Backlog_Requerimientos_Control_Horario_Cafeteria.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="205">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="206">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -641,6 +641,9 @@
   </si>
   <si>
     <t xml:space="preserve">Verificado en vivo tras corregir el bug de semanas superpuestas: el reporte de julio ya muestra correctamente las horas trabajadas y el ajuste de Ana. Se agregó la liquidación mensual y el detalle diario por empleado (8 tests unitarios nuevos en monthly-math.test.ts); falta descargar un reporte real y confirmar visualmente ambas secciones nuevas. Ver ESTADO_PRUEBAS.md.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/marcar activa la cámara (html5-qrcode), valida el QR contra el token activo y registra la marca en /api/time-entries/mark. Verificado en vivo en producción (Vercel, HTTPS): acceso a cámara y marcado real de entrada/salida desde el celular funcionando correctamente. Ver ESTADO_PRUEBAS.md.</t>
   </si>
 </sst>
 </file>
@@ -1232,7 +1235,7 @@
         <v>154</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>165</v>
+        <v>205</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Actualizar seguimiento de RF-08 con el horario por defecto obligatorio
Marca RF-08 como pendiente de reconfirmar en vivo ahora que el alta de
empleado exige cargar el horario por defecto validado contra las
horas semanales pactadas.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Backlog_Requerimientos_Control_Horario_Cafeteria.xlsx
+++ b/Backlog_Requerimientos_Control_Horario_Cafeteria.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="207">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -644,6 +644,9 @@
   </si>
   <si>
     <t xml:space="preserve">/marcar activa la cámara (html5-qrcode), valida el QR contra el token activo y registra la marca en /api/time-entries/mark. Verificado en vivo en producción (Vercel, HTTPS): acceso a cámara y marcado real de entrada/salida desde el celular funcionando correctamente. Ver ESTADO_PRUEBAS.md.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verificado en vivo desde la app real: alta de empleado, generación de usuario e invitación por correo confirmadas. Se agregó el campo obligatorio "Valor hora nominal" (migración 0003_employee_hourly_rate.sql, ya aplicada a la base real). El alta ahora también exige cargar el horario por defecto (RF-09) en el mismo formulario, validando que la suma de horas coincida exactamente con las horas semanales pactadas — si no coincide, se rechaza el alta con un mensaje explícito. Falta reconfirmar en vivo el alta con estos dos campos — ver ESTADO_PRUEBAS.md.</t>
   </si>
 </sst>
 </file>
@@ -1350,7 +1353,7 @@
         <v>154</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="90.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Actualizar seguimiento de RF-08/RF-16 con horas de contrato
Marca ambos como pendientes de reconfirmar en vivo ahora que el alta
de empleado pide horas de contrato y la liquidacion del reporte mide
las horas extra contra ese valor en vez de las horas pactadas.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Backlog_Requerimientos_Control_Horario_Cafeteria.xlsx
+++ b/Backlog_Requerimientos_Control_Horario_Cafeteria.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="211">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -647,6 +647,18 @@
   </si>
   <si>
     <t xml:space="preserve">Verificado en vivo desde la app real: alta de empleado, generación de usuario e invitación por correo confirmadas. Se agregó el campo obligatorio "Valor hora nominal" (migración 0003_employee_hourly_rate.sql, ya aplicada a la base real). El alta ahora también exige cargar el horario por defecto (RF-09) en el mismo formulario, validando que la suma de horas coincida exactamente con las horas semanales pactadas — si no coincide, se rechaza el alta con un mensaje explícito. Falta reconfirmar en vivo el alta con estos dos campos — ver ESTADO_PRUEBAS.md.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El dueño puede crear, editar y desactivar empleados. Al crear un empleado, debe ingresar: nombre completo, cédula, teléfono de contacto, mutualista, contacto de emergencia y correo electrónico (obligatorio, utilizado para el acceso y las comunicaciones del sistema), además de sus horas semanales de contrato, sus horas semanales pactadas (pueden ser menores o mayores al contrato), su valor hora nominal (obligatorio, usado para calcular la liquidación mensual) y un horario por defecto (días/horas) que debe sumar exactamente las horas pactadas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verificado en vivo desde la app real: alta de empleado, generación de usuario e invitación por correo confirmadas. Se agregaron los campos obligatorios "Valor hora nominal" y "Horas semanales de contrato" (independiente de las pactadas), y el horario por defecto obligatorio validado contra las horas pactadas. Falta reconfirmar en vivo el campo de horas de contrato — ver ESTADO_PRUEBAS.md.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El sistema genera un reporte descargable (Excel) por empleado y consolidado, con horas trabajadas, saldos semanales, ajustes manuales aplicados y totales del mes, listo para liquidación de haberes. Incluye el cálculo de la liquidación mensual: las horas extra se calculan contra las horas de CONTRATO del empleado (no contra las pactadas, que pueden ser menores o mayores) — horas hasta el contrato a valor simple, excedente pagado al doble, con las "horas extras que se están pagando" explícitas. Cada hoja de empleado también tiene un detalle diario de entrada/salida/horas trabajadas además del resumen semanal.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verificado en vivo: reporte semanal/consolidado, liquidación con valor hora nominal y detalle diario confirmados. Se redefinió el cálculo de horas extra para que se midan contra las horas de contrato (no las pactadas) — nuevo test en monthly-math.test.ts; falta descargar un reporte real y confirmar visualmente el cambio. Ver ESTADO_PRUEBAS.md.</t>
   </si>
 </sst>
 </file>
@@ -1341,7 +1353,7 @@
         <v>35</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>10</v>
@@ -1353,7 +1365,7 @@
         <v>154</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="90.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1525,7 +1537,7 @@
         <v>59</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>203</v>
+        <v>209</v>
       </c>
       <c r="D17" s="5" t="s">
         <v>10</v>
@@ -1537,7 +1549,7 @@
         <v>154</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>